<commit_message>
Entretoises en tube 20 x 2, serrage des M10 a 25 N.m
- ENTRETOISE_DI 11 -> 16 (cadre et chape) ; COUPLE_M10 = 25 N.m et K_COUPLE
  passent dans params.py, precharge 12,5 kN, soit 111 MPa dans le tube.
- verifie() controle la precharge contre le Re du tube a chaud (190 / 1,5).
- Voilement recalcule (fem_flamb3) : 38,2 couche, 38,3 debout (39,0 / 39,1
  avec le 20 x 4,5). Compression des entretoises de chape : 24,5 MPa.
- DEBOUT, README, REPRISE a jour ; make.py : 0 etape en echec.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -564,7 +564,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Entretoises** : E235+C EN 10305-1, tube de precision 20 x 4,5 ; 9 coupees a 60 +0,1/0 et 2 a 71,5 +/-0,2, faces dressees // 0,05 : ce sont elles qui fixent l ecart des flancs.</t>
+          <t>Entretoises** : E235+C EN 10305-1, tube de precision 20 x 2 ; 9 coupees a 60 +0,1/0 et 2 a 71,5 +/-0,2, faces dressees // 0,05 : ce sont elles qui fixent l ecart des flancs.</t>
         </is>
       </c>
     </row>
@@ -922,11 +922,11 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>tube de precision 20 x 4,5</t>
+          <t>tube de precision 20 x 2</t>
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0.123</v>
+        <v>0.063</v>
       </c>
       <c r="G11" s="7">
         <f>C11*F11</f>
@@ -1033,11 +1033,11 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>tube de precision 20 x 4,5</t>
+          <t>tube de precision 20 x 2</t>
         </is>
       </c>
       <c r="F14" s="7" t="n">
-        <v>0.103</v>
+        <v>0.053</v>
       </c>
       <c r="G14" s="7">
         <f>C14*F14</f>
@@ -1410,7 +1410,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Masse du cadre complet : 35.3 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 05/10/2026).</t>
+          <t>Masse du cadre complet : 34.7 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 05/10/2026).</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>entretoises de cadre : 4 de coin, 2 de bielle, 1 de sommet. Serrage 80 : l ecrou tombe sur le filet avec 6 de marge, la vis en depasse de 10 ; 35 N.m. Pas d ecrou a bague polyamide (ISO 7040, DIN 985) : elle ne freine plus a 150 C. Acier, pas inox : meme dilatation que les flancs, la precharge tient a chaud</t>
+          <t>entretoises de cadre : 4 de coin, 2 de bielle, 1 de sommet. Serrage 80 : l ecrou tombe sur le filet avec 6 de marge, la vis en depasse de 10 ; 25 N.m. Pas d ecrou a bague polyamide (ISO 7040, DIN 985) : elle ne freine plus a 150 C. Acier, pas inox : meme dilatation que les flancs, la precharge tient a chaud</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>vis de chape : tete et 1 rondelle derriere le flanc oppose, flanc, entretoise de cadre, flanc, entretoise de butee, platines, 4 rondelles, ecrou serre puis contre-ecrou bloque contre lui. Serrage 173,5, filet a partir de 168 : le premier ecrou y tombe avec 5,5 de marge, la vis depasse du contre-ecrou de 9,7 ; 35 N.m sur le premier</t>
+          <t>vis de chape : tete et 1 rondelle derriere le flanc oppose, flanc, entretoise de cadre, flanc, entretoise de butee, platines, 4 rondelles, ecrou serre puis contre-ecrou bloque contre lui. Serrage 173,5, filet a partir de 168 : le premier ecrou y tombe avec 5,5 de marge, la vis depasse du contre-ecrou de 9,7 ; 25 N.m sur le premier</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>35 N.m</t>
+          <t>25 N.m</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2410,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>facteur critique 39.0 couche, 39.1 debout (les deux flancs penchent ensemble, tenus par la flexion des 9 entretoises tubulaires, bouts serres)</t>
+          <t>facteur critique 38.2 couche, 38.3 debout (les deux flancs penchent ensemble, tenus par la flexion des 9 entretoises tubulaires, bouts serres)</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Chape. Enfiler sur les deux vis V9 les entretoises de butee de 71,5, puis le sous-ensemble de chape, la tige passant par la fente du coin ; 4 rondelles et un ecrou H par vis, 35 N.m, puis le contre-ecrou H bloque contre lui en tenant le premier.</t>
+          <t>Chape. Enfiler sur les deux vis V9 les entretoises de butee de 71,5, puis le sous-ensemble de chape, la tige passant par la fente du coin ; 4 rondelles et un ecrou H par vis, 25 N.m, puis le contre-ecrou H bloque contre lui en tenant le premier.</t>
         </is>
       </c>
     </row>
@@ -2667,7 +2667,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Pieds. Dresser le cadre et le poser dans ses deux pieds couches, encoche dans encoche : les nodes serrent de 0,1 par cote, chasser au maillet. Bloquer les V1 a 35 N.m. La poutrelle, sans patins, repose sur les bossages.</t>
+          <t>Pieds. Dresser le cadre et le poser dans ses deux pieds couches, encoche dans encoche : les nodes serrent de 0,1 par cote, chasser au maillet. Bloquer les V1 a 25 N.m. La poutrelle, sans patins, repose sur les bossages.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Patin de charge bombe R1000 : vraie flexion 3 points
Dessus du patin de charge en cylindre d'axe transversal, R1000, sommet au
milieu (1,25 de chute aux bords) ; dessous plat, toujours colle. Le plateau
bas du poussoir y porte sur une ligne : Hertz 88 MPa a 12 kN, coefficient
5,4, controle dans verifie(). Vue de face cotee sur la planche 04, note de
fabrication, SPEC (bombe et alignement du poussoir par les goupilles).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1.453</v>
+        <v>1.455</v>
       </c>
       <c r="G7" s="7">
         <f>C7*F7</f>
@@ -786,7 +786,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>dessus a 12 degres sur toute la section ; alesage 25,4 prof. 20 par dessous ; 4 taraudages M8 prof. 16 dans les faces laterales (avant-trou 6,8 prof. 19), axe a 12 du dessous, x = +/- 44</t>
+          <t>dessus a 12 degres sur toute la section ; alesage 25 H8 prof. 20 par dessous ; 4 taraudages M8 prof. 16 dans les faces laterales (avant-trou 6,8 prof. 19), axe a 12 du dessous, x = +/- 44</t>
         </is>
       </c>
     </row>
@@ -811,11 +811,11 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>rond etire 25 h9 x 76</t>
+          <t>rond etire 25 h9 x 79.5</t>
         </is>
       </c>
       <c r="F8" s="7" t="n">
-        <v>0.293</v>
+        <v>0.306</v>
       </c>
       <c r="G8" s="7">
         <f>C8*F8</f>
@@ -823,7 +823,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>rond etire h9 NON repris : tronconne, chanfrein 1,5 x 45 deg aux deux bouts ; flottant, centre la pile et enfile le poussoir et le coulisseau</t>
+          <t>rond etire h9 NON repris : tronconne, chanfrein 1,5 x 45 deg aux deux bouts ; COLLE au fond de l alesage du coulisseau (Loctite 648 (tient 175 C), alesage 25 H8 degraisse) ; centre la pile et coulisse dans le poussoir : 7,9 au repos, 4,3 de garde au dessus du patin a la butee</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
         </is>
       </c>
       <c r="F13" s="7" t="n">
-        <v>0.772</v>
+        <v>0.742</v>
       </c>
       <c r="G13" s="7">
         <f>C13*F13</f>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>DXF = 2 avant-trous 6 a +/- 35, PERCES ET ALESES 8 H7 apres decoupe (goupilles 8 m6 serrees) ; colle en place en meme temps que les patins d appui ; un par eprouvette</t>
+          <t>DXF = 2 avant-trous 6 a +/- 35, PERCES ET ALESES 8 H7 apres decoupe (goupilles 8 m6 serrees) ; dessus BOMBE R1000 fraise (cylindre d axe transversal, 10 au milieu, 8,75 aux bords) : le poussoir y porte sur une ligne ; dessous plat, colle en place en meme temps que les patins d appui ; un par eprouvette</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1410,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Masse du cadre complet : 34.7 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 05/10/2026).</t>
+          <t>Masse du cadre complet : 34.7 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 06/10/2026).</t>
         </is>
       </c>
     </row>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Tete de charge. Encoller le patin de charge sur sa face inferieure et le poser au milieu de la poutrelle, goupilles vers la tete ; enfiler sur les goupilles les 3 plateaux du poussoir, poser la cale eventuelle (V4), le tourillon, la pile TETE-BECHE (grand diametre aux deux bouts) et le coulisseau, cote epais de sa pente vers la chape. De cet encollage a la precharge, tout doit tenir dans la vie en pot de la colle : faire d abord les etapes 2 a 5 et preparer la visserie. Si elle est trop courte, coller le patin de charge la veille sur la poutrelle, centre au trace, sous une masse.</t>
+          <t>Tete de charge. Encoller le patin de charge sur sa face inferieure et le poser au milieu de la poutrelle, goupilles vers la tete ; enfiler sur les goupilles les 3 plateaux du poussoir, poser la cale eventuelle (V4), la pile TETE-BECHE (grand diametre aux deux bouts) puis le coulisseau, tourillon colle dessous a l avance (Loctite 648 dans l alesage degraisse, polymeriser avant montage), cote epais de sa pente vers la chape. De cet encollage a la precharge, tout doit tenir dans la vie en pot de la colle : faire d abord les etapes 2 a 5 et preparer la visserie. Si elle est trop courte, coller le patin de charge la veille sur la poutrelle, centre au trace, sous une masse.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Poussoir visse en bloc, patin de charge raccourci a 58 sans trou
- Les 3 plateaux sont tenus par 2 vis H M6 x 35 (tete dessous, 6 de garde
  a la poutrelle) + rondelle + ecrou ISO 7042 dessus, a x = +/- 38 (trous
  laser 6,6) ; les goupilles 8 m6 et les trous 8 H7 du patin disparaissent.
- Patin de charge 58 x 100 (longueur derivee des tetes de vis), sans trou,
  bombe R1000 (9,58 aux bords) ; 2,07 MPa sur le beton.
- Le poussoir est centre par le tourillon, le patin colle au trace.
- Controles des gardes dans verifie() ; planches 00, 02, 04, nomenclature
  (V3), ordre de montage, SPEC, README, DEBOUT, SUITE a jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="F6" s="7" t="n">
-        <v>0.323</v>
+        <v>0.325</v>
       </c>
       <c r="G6" s="7">
         <f>C6*F6</f>
@@ -749,7 +749,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>3 plateaux perces : alesage 25,4 traversant ; 2 trous de passage 8,3 decoupes au laser a +/- 35, goupilles 8 m6 x 30 libres, serrees dans le patin de charge qui fait fond</t>
+          <t>3 plateaux perces : alesage 25,4 traversant ; 2 trous de passage 6,6 decoupes au laser a +/- 38 ; assembles en bloc par 2 vis H M6 x 35, tete en dessous, ecrou au dessus, 8 N.m ; le patin de charge fait fond</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
         </is>
       </c>
       <c r="F13" s="7" t="n">
-        <v>0.742</v>
+        <v>0.446</v>
       </c>
       <c r="G13" s="7">
         <f>C13*F13</f>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>DXF = 2 avant-trous 6 a +/- 35, PERCES ET ALESES 8 H7 apres decoupe (goupilles 8 m6 serrees) ; dessus BOMBE R1000 fraise (cylindre d axe transversal, 10 au milieu, 8,75 aux bords) : le poussoir y porte sur une ligne ; dessous plat, colle en place en meme temps que les patins d appui ; un par eprouvette</t>
+          <t>sans trou, 58 de long selon x pour laisser passer les tetes des vis du poussoir ; dessus BOMBE R1000 fraise (cylindre d axe transversal, 10 au milieu, 9,58 aux bords) : le poussoir y porte sur une ligne ; dessous plat, colle centre au trace en meme temps que les patins d appui ; un par eprouvette</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1410,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Masse du cadre complet : 34.7 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 06/10/2026).</t>
+          <t>Masse du cadre complet : 34.4 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 06/10/2026).</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Goupille cylindrique ISO 2338 8 m6 x 30</t>
+          <t>Vis H M6 x 35 ISO 4017 8.8 zinguee + rondelle ISO 7089 M6 + ecrou ISO 7042 M6 classe 8 tout metal</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>reperage des plateaux du poussoir : serrees dans le patin de charge (8 H7, enfoncees de 6), libres dans les trous de 8,3 des plateaux ; partent avec l eprouvette</t>
+          <t>serrent les 3 plateaux du poussoir en un bloc, dans les trous de 6,6 a +/- 38 : TETE EN DESSOUS, rondelle et ecrou au dessus, a cote de la pile. Sous le plateau bas il n y a que les 10 du patin de charge jusqu a la poutrelle : une tete de 4 y tient (6 de garde), un ecrou non. Serrage modere, 8 N.m ; la vis depasse de l ecrou de 3,4 ; restent sur le poussoir</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>a decouper ; DXF = brut, reprise apres decoupe</t>
+          <t>a decouper</t>
         </is>
       </c>
     </row>
@@ -2022,7 +2022,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>- Brut de decoupe : le DXF de la traverse porte 1 mm de surepaisseur sur le chant du bas (fraise ensuite en paquet), celui du patin de charge des avant-trous de 6 (perces et aleses 8 H7 ensuite).</t>
+          <t>- Brut de decoupe : le DXF de la traverse porte 1 mm de surepaisseur sur le chant du bas (fraise ensuite en paquet).</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Patin de charge. Chasser les deux goupilles V3 dans ses trous 8 H7, enfoncees de 6 : elles depassent de 24, la hauteur du poussoir.</t>
+          <t>Poussoir, a l avance. Empiler les 3 plateaux, alesages alignes sur un rond de 25 ; passer les deux vis V3 PAR DESSOUS (tete sous le plateau bas), rondelle et ecrou au dessus, serrer a 8 N.m. Le poussoir est desormais un bloc ; il sert a toutes les eprouvettes.</t>
         </is>
       </c>
     </row>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Tete de charge. Encoller le patin de charge sur sa face inferieure et le poser au milieu de la poutrelle, goupilles vers la tete ; enfiler sur les goupilles les 3 plateaux du poussoir, poser la cale eventuelle (V4), la pile TETE-BECHE (grand diametre aux deux bouts) puis le coulisseau, tourillon colle dessous a l avance (Loctite 648 dans l alesage degraisse, polymeriser avant montage), cote epais de sa pente vers la chape. De cet encollage a la precharge, tout doit tenir dans la vie en pot de la colle : faire d abord les etapes 2 a 5 et preparer la visserie. Si elle est trop courte, coller le patin de charge la veille sur la poutrelle, centre au trace, sous une masse.</t>
+          <t>Tete de charge. Encoller le patin de charge sur sa face inferieure et le poser au milieu de la poutrelle, centre au trace, bombe vers la tete ; poser dessus le poussoir visse (3 plateaux), tetes de vis en bas de part et d autre du patin ; poser la cale eventuelle (V4), la pile TETE-BECHE (grand diametre aux deux bouts) puis le coulisseau, tourillon colle dessous a l avance (Loctite 648 dans l alesage degraisse, polymeriser avant montage), cote epais de sa pente vers la chape. De cet encollage a la precharge, tout doit tenir dans la vie en pot de la colle : faire d abord les etapes 2 a 5 et preparer la visserie. Si elle est trop courte, coller le patin de charge la veille sur la poutrelle, centre au trace, sous une masse.</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2788,7 @@
     <row r="32">
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Les plats, les patins d appui et le patin de charge sont colles sur la poutrelle et partent avec elle : il faut un jeu neuf par eprouvette (4 patins d appui, 1 patin de charge et ses 2 goupilles, 2 plats ; colle). Les goupilles, serrees dans le patin de charge, montent de 24 dans le poussoir, et la tete ne peut remonter que de 9,9 avant que le coulisseau touche les entretoises de chape : l eprouvette ne sort pas cadre ferme, on rouvre le flanc cote chape.</t>
+          <t>Les plats, les patins d appui et le patin de charge sont colles sur la poutrelle et partent avec elle : il faut un jeu neuf par eprouvette (4 patins d appui, 1 patin de charge, 2 plats ; colle). Le poussoir visse porte sur le patin de charge, centre par le tourillon, et la tete ne peut remonter que de 9,9 avant que le coulisseau touche les entretoises de chape : l eprouvette ne sort pas cadre ferme, on rouvre le flanc cote chape.</t>
         </is>
       </c>
     </row>
@@ -2838,7 +2838,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Sortir l eprouvette avec sa tete de charge ; sur l etabli, degager le poussoir des goupilles, qui restent dans le patin de charge.</t>
+          <t>Sortir l eprouvette avec sa tete de charge ; sur l etabli, soulever le poussoir visse, qui resservira tel quel : le patin de charge reste colle sur la poutrelle.</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Remonter la nouvelle eprouvette, preparee aux etapes 1, 3 et 5 de l ordre de montage, en reprenant a l etape 8 : le premier flanc a garde ses vis, ses entretoises et la traverse.</t>
+          <t>Remonter la nouvelle eprouvette, preparee aux etapes 1 et 5 de l ordre de montage, en reprenant a l etape 8 : le premier flanc a garde ses vis, ses entretoises et la traverse.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rondelles Belleville : EN 16983 A50 en 51CrV4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -852,7 +852,7 @@
         </is>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1.373</v>
+        <v>1.377</v>
       </c>
       <c r="G9" s="7">
         <f>C9*F9</f>
@@ -860,7 +860,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>acier taraude M16 sur 80 depuis le bout EPAIS, passage 18 au dela ; porte les deux plaques de frottement du commerce entre rebords de 3 : dessus 7,05, dessous 8,15 (faces normales a la pente)</t>
+          <t>acier taraude M16 sur 80 depuis le bout EPAIS, passage 18 au dela ; porte les deux plaques de frottement du commerce entre rebords de 3 : dessus 6,25, dessous 7,36 (faces normales a la pente)</t>
         </is>
       </c>
     </row>
@@ -1389,12 +1389,12 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>12 rondelles DIN 2093 A50</t>
+          <t>12 rondelles EN 16983 A50</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>51CrV4</t>
+          <t>51CrV4 (1.8159)</t>
         </is>
       </c>
       <c r="F9" s="7" t="n">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>piece du commerce : 12 rondelles 50 x 25,4 x 3 montees TETE-BECHE, grand diametre aux deux bouts ; 18,5 kN a plat, course 15,6 mm ; cales de rattrapage 1 et 2 mm (50 / 26) entre poussoir et pile si l empilement est court</t>
+          <t>piece du commerce : 12 rondelles 50 x 25,4 x 3 (ex-DIN 2093, PAS en C60S) montees TETE-BECHE, grand diametre aux deux bouts ; 18,5 kN a plat, course 15,6 mm ; cales de rattrapage 1 et 2 mm (50 / 26) entre poussoir et pile si l empilement est court</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2122,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>12 x DIN 2093 A50, hauteur libre 51.6 mm</t>
+          <t>12 x EN 16983 A50 en 51CrV4 (1.8159), hauteur libre 51.6 mm</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>7.05 (dessus) et 8.15 (dessous) x 3, 6.5 MPa de flexion, garde 2 sous le bronze</t>
+          <t>6.25 (dessus) et 7.36 (dessous) x 3, 8.3 MPa de flexion, garde 2 sous le bronze</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Flancs : microbillage puis brunissage noir mat
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -557,12 +557,19 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Epaisseurs reelles** : mesurer les deux toles livrees, regler EP_TOLE_REELLE_42 (42CrMo4) et EP_TOLE_REELLE_S355 (S355JR) et regenerer les DXF avant decoupe. Chaque decoupe suit la tole qu elle RECOIT : EP_TOLE_REELLE_S355 (8 aujourd hui) pour les encoches a mi-bois et la mortaise de traverse du flanc et les fentes de calage du pied ; EP_TOLE_REELLE_42 (8) pour les encoches et nodes du pied et les rainures des patins.</t>
+          <t>Finition des flancs** : apres decoupe et aretes cassees : MICROBILLAGE puis BRUNISSAGE noir (oxydation a chaud), aspect mat ; huile de protection legere, ESSUYEE avant la premiere chauffe (elle fume a 150 C) ; traits de graduation repasses a la peinture blanche haute temperature apres brunissage. Noir mat pour la correlation d images, et sans epaisseur : ni les jeux des encoches ni les serrages des entretoises n en dependent. Les autres pieces restent brutes.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Epaisseurs reelles** : mesurer les deux toles livrees, regler EP_TOLE_REELLE_42 (42CrMo4) et EP_TOLE_REELLE_S355 (S355JR) et regenerer les DXF avant decoupe. Chaque decoupe suit la tole qu elle RECOIT : EP_TOLE_REELLE_S355 (8 aujourd hui) pour les encoches a mi-bois et la mortaise de traverse du flanc et les fentes de calage du pied ; EP_TOLE_REELLE_42 (8) pour les encoches et nodes du pied et les rainures des patins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Entretoises** : E235+C EN 10305-1, tube de precision 20 x 2 ; 9 coupees a 60 +0,1/0 et 2 a 71,5 +/-0,2, faces dressees // 0,05 : ce sont elles qui fixent l ecart des flancs.</t>
         </is>
@@ -675,7 +682,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>decoupe laser, aretes cassees 0,8 x 45 deg, bossages non repris ; encoches a mi-bois et mortaise taillees sur la tole REELLE S355 des pieces qu elles recoivent : mesurer les deux toles livrees, regler EP_TOLE_REELLE_42 (42CrMo4) et EP_TOLE_REELLE_S355 (S355JR) et regenerer les DXF avant decoupe ; graduation de charge gravee (calque GRAVURE) d un seul cote de la lumiere, face gravee montee a l exterieur</t>
+          <t>decoupe laser, aretes cassees 0,8 x 45 deg, bossages non repris ; encoches a mi-bois et mortaise taillees sur la tole REELLE S355 des pieces qu elles recoivent : mesurer les deux toles livrees, regler EP_TOLE_REELLE_42 (42CrMo4) et EP_TOLE_REELLE_S355 (S355JR) et regenerer les DXF avant decoupe ; graduation de charge gravee (calque GRAVURE) d un seul cote de la lumiere, face gravee montee a l exterieur ; finition : apres decoupe et aretes cassees : MICROBILLAGE puis BRUNISSAGE noir (oxydation a chaud), aspect mat ; huile de protection legere, ESSUYEE avant la premiere chauffe (elle fume a 150 C) ; traits de graduation repasses a la peinture blanche haute temperature apres brunissage</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Flancs : sablage corindon, huile ester HT, gravure 0,2 mini
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -557,7 +557,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Finition des flancs** : apres decoupe et aretes cassees : MICROBILLAGE puis BRUNISSAGE noir (oxydation a chaud), aspect mat ; huile de protection legere, ESSUYEE avant la premiere chauffe (elle fume a 150 C) ; traits de graduation repasses a la peinture blanche haute temperature apres brunissage. Noir mat pour la correlation d images, et sans epaisseur : ni les jeux des encoches ni les serrages des entretoises n en dependent. Les autres pieces restent brutes.</t>
+          <t>Finition des flancs** : apres decoupe et aretes cassees : SABLAGE corindon des deux faces a l identique, pression moderee (planeite), puis BRUNISSAGE noir (oxydation a chaud), aspect mat ; degraisser l huile de sortie de bain, puis film d huile ESTER synthetique haute temperature passe au chiffon et ESSUYE ; ni huile minerale ni silicone ; graduation gravee a 0.2 de profondeur au moins, traits repasses a la peinture blanche haute temperature apres brunissage. Noir mat pour la correlation d images, et quasi sans epaisseur : ni les jeux des encoches ni les serrages des entretoises n en dependent. Les autres pieces restent brutes.</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>decoupe laser, aretes cassees 0,8 x 45 deg, bossages non repris ; encoches a mi-bois et mortaise taillees sur la tole REELLE S355 des pieces qu elles recoivent : mesurer les deux toles livrees, regler EP_TOLE_REELLE_42 (42CrMo4) et EP_TOLE_REELLE_S355 (S355JR) et regenerer les DXF avant decoupe ; graduation de charge gravee (calque GRAVURE) d un seul cote de la lumiere, face gravee montee a l exterieur ; finition : apres decoupe et aretes cassees : MICROBILLAGE puis BRUNISSAGE noir (oxydation a chaud), aspect mat ; huile de protection legere, ESSUYEE avant la premiere chauffe (elle fume a 150 C) ; traits de graduation repasses a la peinture blanche haute temperature apres brunissage</t>
+          <t>decoupe laser, aretes cassees 0,8 x 45 deg, bossages non repris ; encoches a mi-bois et mortaise taillees sur la tole REELLE S355 des pieces qu elles recoivent : mesurer les deux toles livrees, regler EP_TOLE_REELLE_42 (42CrMo4) et EP_TOLE_REELLE_S355 (S355JR) et regenerer les DXF avant decoupe ; graduation de charge gravee (calque GRAVURE) d un seul cote de la lumiere, face gravee montee a l exterieur ; finition : apres decoupe et aretes cassees : SABLAGE corindon des deux faces a l identique, pression moderee (planeite), puis BRUNISSAGE noir (oxydation a chaud), aspect mat ; degraisser l huile de sortie de bain, puis film d huile ESTER synthetique haute temperature passe au chiffon et ESSUYE ; ni huile minerale ni silicone ; graduation gravee a 0.2 de profondeur au moins, traits repasses a la peinture blanche haute temperature apres brunissage</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plaquettes du coin usinees en CuSn12 : 38 x 102 et 38 x 104 x 5, sans trou
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -586,11 +586,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1.377</v>
+        <v>1.371</v>
       </c>
       <c r="G9" s="7">
         <f>C9*F9</f>
@@ -867,36 +867,36 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>acier taraude M16 sur 80 depuis le bout EPAIS, passage 18 au dela ; porte les deux plaques de frottement du commerce entre rebords de 3 : dessus 6,25, dessous 7,36 (faces normales a la pente)</t>
+          <t>acier taraude M16 sur 80 depuis le bout EPAIS, passage 18 au dela ; porte les deux plaques de frottement en bronze entre rebords de 3 : dessus 5,25, dessous 5,41 (faces normales a la pente)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>06c</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Platine de butee de la vis</t>
+          <t>Plaque de frottement, dessus</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>42CrMo4 +A</t>
+          <t>CuSn12-C</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>tole 8 mm, cert. 3.1, Re &gt;= 430</t>
+          <t>plat 40 x 6</t>
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>0.451</v>
+        <v>0.171</v>
       </c>
       <c r="G10" s="7">
         <f>C10*F10</f>
@@ -904,36 +904,36 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>meme tole 42CrMo4 que les flancs (imbriquees dans leurs chutes), empilees et serrees par les deux vis H M10 x 200 de la chape</t>
+          <t>fraisee 38 x 102 x 5, sans trou, faces planes et paralleles a 0,02, Ra 0,8 cote glissement, aretes cassees 0,3 ; entre ses deux rebords sur le dessus du coin, points de silicone HT au montage ; pate graphite haute temperature sur la face qui glisse sous la traverse</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>07b</t>
+          <t>06d</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Entretoise de butee</t>
+          <t>Plaque de frottement, dessous</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>E235+C EN 10305-1</t>
+          <t>CuSn12-C</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>tube de precision 20 x 2</t>
+          <t>plat 40 x 6</t>
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0.063</v>
+        <v>0.174</v>
       </c>
       <c r="G11" s="7">
         <f>C11*F11</f>
@@ -941,36 +941,36 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>coupee a 71,5 +/-0,2, faces dressees ; en compression pure : c est elle qui porte l effort de commande</t>
+          <t>comme la haute, mais 38 x 104 x 5 ; entre ses deux rebords sous le coin, points de silicone HT au montage ; pate graphite haute temperature sur la face qui glisse sur la pente du coulisseau</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>04a</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Patin d'appui rainure</t>
+          <t>Platine de butee de la vis</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>S355JR</t>
+          <t>42CrMo4 +A</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>tole 10 mm</t>
+          <t>tole 8 mm, cert. 3.1, Re &gt;= 430</t>
         </is>
       </c>
       <c r="F12" s="7" t="n">
-        <v>0.129</v>
+        <v>0.451</v>
       </c>
       <c r="G12" s="7">
         <f>C12*F12</f>
@@ -978,36 +978,36 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>decoupe laser PUIS rainure 9,5 x 1,5 fraisee sur toute la longueur de la face d appui (0,75 de jeu par cote sur la tole reelle du flanc) ; colle en place, cadre monte, sous 0,5 kN de precharge ; un jeu par eprouvette</t>
+          <t>meme tole 42CrMo4 que les flancs (imbriquees dans leurs chutes), empilees et serrees par les deux vis H M10 x 200 de la chape</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>04b</t>
+          <t>07b</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Patin de charge</t>
+          <t>Entretoise de butee</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>S355JR</t>
+          <t>E235+C EN 10305-1</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>tole 10 mm</t>
+          <t>tube de precision 20 x 2</t>
         </is>
       </c>
       <c r="F13" s="7" t="n">
-        <v>0.446</v>
+        <v>0.063</v>
       </c>
       <c r="G13" s="7">
         <f>C13*F13</f>
@@ -1015,36 +1015,36 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>sans trou, 58 de long selon x pour laisser passer les tetes des vis du poussoir ; dessus BOMBE R1000 fraise (cylindre d axe transversal, 10 au milieu, 9,58 aux bords) : le poussoir y porte sur une ligne ; dessous plat, colle centre au trace en meme temps que les patins d appui ; un par eprouvette</t>
+          <t>coupee a 71,5 +/-0,2, faces dressees ; en compression pure : c est elle qui porte l effort de commande</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>06b</t>
+          <t>04a</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Entretoise tubulaire</t>
+          <t>Patin d'appui rainure</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>E235+C EN 10305-1</t>
+          <t>S355JR</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>tube de precision 20 x 2</t>
+          <t>tole 10 mm</t>
         </is>
       </c>
       <c r="F14" s="7" t="n">
-        <v>0.053</v>
+        <v>0.129</v>
       </c>
       <c r="G14" s="7">
         <f>C14*F14</f>
@@ -1052,23 +1052,23 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>coupee a 60 +0,1/0, faces dressees // 0,05 : c est elle qui fixe l ecart des flancs ; 7 serrees par vis TH M10 x 100 + ecrou ISO 7042 classe 8, autofreine tout metal, les 2 de la chape par les vis H M10 x 200</t>
+          <t>decoupe laser PUIS rainure 9,5 x 1,5 fraisee sur toute la longueur de la face d appui (0,75 de jeu par cote sur la tole reelle du flanc) ; colle en place, cadre monte, sous 0,5 kN de precharge ; un jeu par eprouvette</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>04b</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Pied a mi-bois</t>
+          <t>Patin de charge</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
@@ -1077,11 +1077,11 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>tole 8 mm, cert. 2.2</t>
+          <t>tole 10 mm</t>
         </is>
       </c>
       <c r="F15" s="7" t="n">
-        <v>0.87</v>
+        <v>0.446</v>
       </c>
       <c r="G15" s="7">
         <f>C15*F15</f>
@@ -1089,36 +1089,36 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>ajoure, bossages aux deux bouts qui posent sur les crochets d etuve, fente de calage 8,4 x 7 a 5 du bout ; encoches et nodes taillees sur la tole REELLE du flanc (42CrMo4), fente sur celle du crochet (S355) : mesurer les deux toles livrees, regler EP_TOLE_REELLE_42 (42CrMo4) et EP_TOLE_REELLE_S355 (S355JR) et regenerer les DXF avant decoupe ; meme plaque pour les deux positions : 2 dans le chant bas (couche), 2 aux coins de l about a 38 degres (debout), aretes de pose a 447</t>
+          <t>sans trou, 58 de long selon x pour laisser passer les tetes des vis du poussoir ; dessus BOMBE R1000 fraise (cylindre d axe transversal, 10 au milieu, 9,58 aux bords) : le poussoir y porte sur une ligne ; dessous plat, colle centre au trace en meme temps que les patins d appui ; un par eprouvette</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>05c</t>
+          <t>06b</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Crochet d etuve</t>
+          <t>Entretoise tubulaire</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>S355JR</t>
+          <t>E235+C EN 10305-1</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>tole 8 mm, cert. 2.2</t>
+          <t>tube de precision 20 x 2</t>
         </is>
       </c>
       <c r="F16" s="7" t="n">
-        <v>0.173</v>
+        <v>0.053</v>
       </c>
       <c r="G16" s="7">
         <f>C16*F16</f>
@@ -1126,26 +1126,100 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
+          <t>coupee a 60 +0,1/0, faces dressees // 0,05 : c est elle qui fixe l ecart des flancs ; 7 serrees par vis TH M10 x 100 + ecrou ISO 7042 classe 8, autofreine tout metal, les 2 de la chape par les vis H M10 x 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Pied a mi-bois</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>S355JR</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>tole 8 mm, cert. 2.2</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G17" s="7">
+        <f>C17*F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>ajoure, bossages aux deux bouts qui posent sur les crochets d etuve, fente de calage 8,4 x 7 a 5 du bout ; encoches et nodes taillees sur la tole REELLE du flanc (42CrMo4), fente sur celle du crochet (S355) : mesurer les deux toles livrees, regler EP_TOLE_REELLE_42 (42CrMo4) et EP_TOLE_REELLE_S355 (S355JR) et regenerer les DXF avant decoupe ; meme plaque pour les deux positions : 2 dans le chant bas (couche), 2 aux coins de l about a 38 degres (debout), aretes de pose a 447</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>05c</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Crochet d etuve</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>S355JR</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>tole 8 mm, cert. 2.2</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>0.173</v>
+      </c>
+      <c r="G18" s="7">
+        <f>C18*F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
           <t>cadre DEBOUT : pend par 4 langues a bec dans la colonne de trous carres de 10 (paroi 1), dans le plan des flancs ; l arete du pied en V pose sur son appui, calee par la dent dans la fente du pied. Le fond de l etuve ne porte rien ; dent a 47,2 de la paroi pour une etuve de 538</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="8" t="n"/>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="8" t="n"/>
-      <c r="F17" s="9" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="8" t="n"/>
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>total</t>
         </is>
       </c>
-      <c r="G17" s="10">
-        <f>SUM(G4:G16)</f>
+      <c r="G19" s="10">
+        <f>SUM(G4:G18)</f>
         <v/>
       </c>
-      <c r="H17" s="8" t="n"/>
+      <c r="H19" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1158,14 +1232,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
     <col width="33" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
   </cols>
@@ -1251,12 +1325,12 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>06c</t>
+          <t>02d</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Plaque de frottement, dessus</t>
+          <t>Tige filetee de commande M16</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
@@ -1264,65 +1338,65 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>norelem 23765-01-038100, 38 x 100 x 5</t>
+          <t>tige filetee M16 classe 8.8, coupee a 185</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>CuZn25Al5Mn4Fe3-C + graphite</t>
+          <t>8.8</t>
         </is>
       </c>
       <c r="F5" s="7" t="n">
-        <v>0.148</v>
+        <v>0.407</v>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>piece du commerce, autolubrifiante ; entre ses deux rebords sur le dessus du coin, trous remplis de silicone HT, glisse sous la traverse</t>
+          <t>piece du commerce, coupee a longueur, montee a la pate cuivre ; ecrous et butee figures : ils montrent l arret axial dans les deux sens</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>06d</t>
+          <t>04c</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Plaque de frottement, dessous</t>
+          <t>Plat de renfort colle</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>norelem 23765-01-038100, 38 x 100 x 5</t>
+          <t>feuillard 20 x 2 S235, coupe a 840</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>CuZn25Al5Mn4Fe3-C + graphite</t>
+          <t>S235</t>
         </is>
       </c>
       <c r="F6" s="7" t="n">
-        <v>0.148</v>
+        <v>0.26</v>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>meme plaque du commerce ; entre ses deux rebords sous le coin, trous remplis de silicone HT, glisse sur la pente du coulisseau</t>
+          <t>piece du commerce, coupee a longueur, bavures retirees ; collee sur toute la longueur a y = +/- 34, poncer et degraisser les deux faces ; un jeu par eprouvette</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>02d</t>
+          <t>02e</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Tige filetee de commande M16</t>
+          <t>Pile de 12 rondelles Belleville</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
@@ -1330,94 +1404,28 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>tige filetee M16 classe 8.8, coupee a 185</t>
+          <t>12 rondelles EN 16983 A50</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>8.8</t>
+          <t>51CrV4 (1.8159)</t>
         </is>
       </c>
       <c r="F7" s="7" t="n">
-        <v>0.407</v>
+        <v>0.412</v>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>piece du commerce, coupee a longueur, montee a la pate cuivre ; ecrous et butee figures : ils montrent l arret axial dans les deux sens</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>04c</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Plat de renfort colle</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>feuillard 20 x 2 S235, coupe a 840</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>S235</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>piece du commerce, coupee a longueur, bavures retirees ; collee sur toute la longueur a y = +/- 34, poncer et degraisser les deux faces ; un jeu par eprouvette</t>
-        </is>
-      </c>
-    </row>
+          <t>piece du commerce : 12 rondelles 50 x 25,4 x 3 (ex-DIN 2093, PAS en C60S) montees TETE-BECHE, grand diametre aux deux bouts ; 18,5 kN a plat, course 15,6 mm ; cales de rattrapage 1 et 2 mm (50 / 26) entre poussoir et pile si l empilement est court</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>02e</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Pile de 12 rondelles Belleville</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>12 rondelles EN 16983 A50</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>51CrV4 (1.8159)</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>0.412</v>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>piece du commerce : 12 rondelles 50 x 25,4 x 3 (ex-DIN 2093, PAS en C60S) montees TETE-BECHE, grand diametre aux deux bouts ; 18,5 kN a plat, course 15,6 mm ; cales de rattrapage 1 et 2 mm (50 / 26) entre poussoir et pile si l empilement est court</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Masse du cadre complet : 34.4 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 06/10/2026).</t>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Masse du cadre complet : 34.4 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 07/10/2026).</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2305,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>norelem 23765-01-038100, 38 x 100 x 5, CuZn25Al5Mn4Fe3-C + graphite ; 7.7 MPa au plus pour 35 admis</t>
+          <t>usinees en CuSn12-C, 38 x 102 (dessus) et 38 x 104 (dessous) x 5 ; pate graphite haute temperature ; 7.6 MPa au plus pour 25 admis</t>
         </is>
       </c>
     </row>
@@ -2309,7 +2317,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>6.25 (dessus) et 7.36 (dessous) x 3, 8.3 MPa de flexion, garde 2 sous le bronze</t>
+          <t>5.25 (dessus) et 5.41 (dessous) x 3, 11.8 MPa de flexion, garde 2 sous le bronze</t>
         </is>
       </c>
     </row>
@@ -2321,7 +2329,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>30.0 x 51.8 mm (sur 60) en fin de course, 7.7 MPa</t>
+          <t>30.0 x 52.8 mm (sur 60) en fin de course, 7.6 MPa</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2341,7 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>38.0 x 48.6 mm (sur 58) en fin de course, 6.5 MPa</t>
+          <t>38.0 x 50.6 mm (sur 58) en fin de course, 6.2 MPa</t>
         </is>
       </c>
     </row>
@@ -2574,7 +2582,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Coin, a l avance. Degraisser les deux sieges ; poser chaque plaque de frottement ENTRE SES DEUX REBORDS, trous remplis et quelques points de silicone haute temperature -- PAS d epoxy, bronze et acier ne se dilatent pas pareil ; laisser prendre. Aucune pate sur les plaques ni sur les sieges : elles sont autolubrifiantes, et le silicone ne prend pas sur une pate.</t>
+          <t>Coin, a l avance. Degraisser les deux sieges ; poser chaque plaque de frottement ENTRE SES DEUX REBORDS (la plus longue, 104, dessous), quelques points de silicone haute temperature sur le siege degraisse -- PAS d epoxy, bronze et acier ne se dilatent pas pareil ; laisser prendre. PUIS seulement, pate graphite haute temperature sur les faces de glissement, rien sur les sieges : le silicone ne prend pas sur une pate.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Commande : vis H M16 x 160 ISO 4017 filetage total au lieu de la tige et des ecrous de tete
Visserie renumerotee : V8 -> V7, V9 -> V8.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -1238,7 +1238,7 @@
     <col width="70" customWidth="1" min="1" max="1"/>
     <col width="33" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="63" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Tige filetee de commande M16</t>
+          <t>Vis de commande H M16 x 160</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>tige filetee M16 classe 8.8, coupee a 185</t>
+          <t>vis H M16 x 160 ISO 4017 8.8 zinguee, filetee jusqu a la tete</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -1347,11 +1347,11 @@
         </is>
       </c>
       <c r="F5" s="7" t="n">
-        <v>0.407</v>
+        <v>0.353</v>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>piece du commerce, coupee a longueur, montee a la pate cuivre ; ecrous et butee figures : ils montrent l arret axial dans les deux sens</t>
+          <t>piece du commerce, filetee jusqu a la tete, montee a la pate cuivre ; tete de 10 (douille de 24) sur la butee ; ecrous et butee figures : ils montrent l arret axial dans les deux sens</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>cote interieur des platines, sous les ecrous V8 : deux empilees font les 2 mm de rondelle trempee (une rondelle trempee 30 x 2 n existe pas en M16)</t>
+          <t>cote interieur des platines, sous les ecrous V7 : deux empilees font les 2 mm de rondelle trempee (une rondelle trempee 30 x 2 n existe pas en M16)</t>
         </is>
       </c>
     </row>
@@ -1607,15 +1607,15 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Ecrou M16 H ISO 4032 classe 8 + ecrou M16 HM ISO 4035, bloques</t>
+          <t>Ecrou M16 HM ISO 4035</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>tete de manoeuvre, 22,8 de haut, en appui sur la butee a aiguilles. Douille de 24 et cliquet : une cle plate bute sur les bouts des vis V9</t>
+          <t>bloques l un sur l autre cote interieur des platines, sur les rondelles V5, avec 0,1 a 0,3 de jeu axial : ils ne retiennent la vis qu au desserrage, 329 N</t>
         </is>
       </c>
     </row>
@@ -1627,33 +1627,13 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Ecrou M16 HM ISO 4035</t>
+          <t>Vis H M10 x 200 ISO 4014 8.8 zinguee (filetee sur 32) + 2 ecrous H M10 ISO 4032 classe 8 + 5 rondelles ISO 7089 M10</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>bloques l un sur l autre cote interieur des platines, sur les rondelles V5, avec 0,1 a 0,3 de jeu axial : ils ne retiennent la tige qu au desserrage, 329 N</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>V9</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Vis H M10 x 200 ISO 4014 8.8 zinguee (filetee sur 32) + 2 ecrous H M10 ISO 4032 classe 8 + 5 rondelles ISO 7089 M10</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>vis de chape : tete et 1 rondelle derriere le flanc oppose, flanc, entretoise de cadre, flanc, entretoise de butee, platines, 4 rondelles, ecrou serre puis contre-ecrou bloque contre lui. Serrage 173,5, filet a partir de 168 : le premier ecrou y tombe avec 5,5 de marge, la vis depasse du contre-ecrou de 9,7 ; 25 N.m sur le premier</t>
         </is>
@@ -2233,7 +2213,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>0.84 tour de tige apres le contact (0.36 mm de pile, 1.7 mm de coin)</t>
+          <t>0.84 tour de vis apres le contact (0.36 mm de pile, 1.7 mm de coin)</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2232,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Couple de serrage des vis M10 (V1, V9)</t>
+          <t>Couple de serrage des vis M10 (V1, V8)</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -2602,7 +2582,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Sous-ensemble de chape, sur l etabli. Sur la tige M16, visser par son bout exterieur l ecrou H et l ecrou HM de manoeuvre (V7), bloques a 2,7 du bout ; enfiler par l autre bout une rondelle AS, la butee AXK 1730 et la seconde AS (V6), les deux platines, les deux rondelles trempees (V5), puis visser les deux ecrous HM (V8) : 0,1 a 0,3 mm de jeu axial, contre-bloquer. Pate cuivre sur le filet de la tige.</t>
+          <t>Sous-ensemble de chape, sur l etabli. Sur la vis H M16 x 160 (02d), enfiler sous la tete une rondelle AS, la butee AXK 1730 et la seconde AS (V6), les deux platines, les deux rondelles trempees (V5), puis visser les deux ecrous HM (V7) : 0,1 a 0,3 mm de jeu axial, contre-bloquer. Pate cuivre sur le filet de la vis.</t>
         </is>
       </c>
     </row>
@@ -2622,7 +2602,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Premier flanc. Poser a plat, sur cales de 20, le flanc OPPOSE a la chape, face gravee DESSOUS : la graduation doit finir a l exterieur. Passer par dessous, rondelle sous tete, les 7 vis V1 (4 de coin, 2 de bielle, 1 de sommet) et les 2 vis V9 (chape, x = +/- 52). Enfiler une entretoise de 60 sur chacune des 9 vis.</t>
+          <t>Premier flanc. Poser a plat, sur cales de 20, le flanc OPPOSE a la chape, face gravee DESSOUS : la graduation doit finir a l exterieur. Passer par dessous, rondelle sous tete, les 7 vis V1 (4 de coin, 2 de bielle, 1 de sommet) et les 2 vis V8 (chape, x = +/- 52). Enfiler une entretoise de 60 sur chacune des 9 vis.</t>
         </is>
       </c>
     </row>
@@ -2672,7 +2652,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Chape. Enfiler sur les deux vis V9 les entretoises de butee de 71,5, puis le sous-ensemble de chape, la tige passant par la fente du coin ; 4 rondelles et un ecrou H par vis, 25 N.m, puis le contre-ecrou H bloque contre lui en tenant le premier.</t>
+          <t>Chape. Enfiler sur les deux vis V8 les entretoises de butee de 71,5, puis le sous-ensemble de chape, la vis passant par la fente du coin ; 4 rondelles et un ecrou H par vis, 25 N.m, puis le contre-ecrou H bloque contre lui en tenant le premier.</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2692,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Coin. Pate cuivre dans son taraudage ; l engager du cote des tetes de V9, bout MINCE en premier, par la fente du flanc, entre la traverse et le coulisseau ; visser la tige jusqu au contact. Le bout epais doit alors etre a moins de 5 mm de sa position de repos, 47,5 mm hors de la face exterieure du flanc ; sinon revoir les cales (etape 5).</t>
+          <t>Coin. Pate cuivre dans son taraudage ; l engager du cote des tetes de V8, bout MINCE en premier, par la fente du flanc, entre la traverse et le coulisseau ; visser la vis jusqu au contact. Le bout epais doit alors etre a moins de 5 mm de sa position de repos, 47,5 mm hors de la face exterieure du flanc ; sinon revoir les cales (etape 5).</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2702,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Precharge. 0,84 tour de tige au dela du contact (0,36 mm de pile, 1,7 mm de coin) donne 0,5 kN. Laisser polymeriser sous cette precharge : l epoxy rattrape l hyperstaticite des quatre appuis. Post-cuire selon la notice Duralco avant toute mise en charge.</t>
+          <t>Precharge. 0,84 tour de vis au dela du contact (0,36 mm de pile, 1,7 mm de coin) donne 0,5 kN. Laisser polymeriser sous cette precharge : l epoxy rattrape l hyperstaticite des quatre appuis. Post-cuire selon la notice Duralco avant toute mise en charge.</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2759,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>L entrer dans l etuve tige vers la porte, pieds tenus 5 mm au dessus des appuis jusqu au fond, puis descendre les quatre fentes des pieds sur les dents des crochets.</t>
+          <t>L entrer dans l etuve vis vers la porte, pieds tenus 5 mm au dessus des appuis jusqu au fond, puis descendre les quatre fentes des pieds sur les dents des crochets.</t>
         </is>
       </c>
     </row>
@@ -2813,7 +2793,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Decharger : devisser la tige jusqu a liberer la pile, puis jusqu a degager le filet ; sortir le coin du cote des tetes de V9.</t>
+          <t>Decharger : devisser la vis jusqu a liberer la pile, puis jusqu a degager le filet ; sortir le coin du cote des tetes de V8.</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2813,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Deposer les ecrous et rondelles des deux V9, le sous-ensemble de chape d un bloc (platines et tige), puis les deux entretoises de butee.</t>
+          <t>Deposer les ecrous et rondelles des deux V8, le sous-ensemble de chape d un bloc (platines et vis), puis les deux entretoises de butee.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Vis de commande M16 en 8.8 brute
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -1238,7 +1238,7 @@
     <col width="70" customWidth="1" min="1" max="1"/>
     <col width="33" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="63" customWidth="1" min="4" max="4"/>
+    <col width="61" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>vis H M16 x 160 ISO 4017 8.8 zinguee, filetee jusqu a la tete</t>
+          <t>vis H M16 x 160 ISO 4017 8.8 brute, filetee jusqu a la tete</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Paquet de traverse : deux vis H M10 x 80 filetage total au lieu d'une tige filetee
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="F5" s="7" t="n">
-        <v>0.256</v>
+        <v>0.25</v>
       </c>
       <c r="G5" s="7">
         <f>C5*F5</f>
@@ -1507,15 +1507,15 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Tige filetee M10 x 90 classe 8.8 + 2 rondelles ISO 7089 M10 + 2 ecrous ISO 7042 classe 8, autofreine tout metal</t>
+          <t>Vis H M10 x 80 ISO 4017 8.8 zinguee (filetage total) + ecrou ISO 7042 classe 8, autofreine tout metal + 2 rondelles ISO 7089 M10</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>tirant du paquet de plaques de traverse, ne reprend aucune charge. Serrage 52, depasse de 9 a chaque bout. Tole mesuree au dela de 10 : prendre une M10 x 100 (verifie() le signale)</t>
+          <t>paquet de plaques de traverse, a y = +/- 17 : les deux vis tiennent les plaques alignees pour dresser le chant en paquet ; elles ne reprennent aucune charge. Serrage 52, la vis depasse de l ecrou de 18 ; 25 N.m. Tole mesuree au dela de 10,5 : prendre des M10 x 90 (verifie() le signale)</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Traverse. Engager dans la mortaise le paquet des 6 plaques, serre par la tige V2 (rondelles et ecrous ISO 7042) ; chants fraises du cote du coin.</t>
+          <t>Traverse. Engager dans la mortaise le paquet des 6 plaques, serre par les deux vis V2 (rondelle sous tete et sous ecrou ISO 7042, 25 N.m) ; chants dresses du cote du coin.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V1 et V2 : meme vis TH M10 x 100 ISO 4017 a filetage total
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -1487,7 +1487,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Vis TH M10 x 100 ISO 4014 8.8 zinguee + ecrou ISO 7042 classe 8, autofreine tout metal + 2 rondelles ISO 7089 M10</t>
+          <t>Vis TH M10 x 100 ISO 4017 8.8 zinguee (filetage total) + ecrou ISO 7042 classe 8, autofreine tout metal + 2 rondelles ISO 7089 M10</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>entretoises de cadre : 4 de coin, 2 de bielle, 1 de sommet. Serrage 80 : l ecrou tombe sur le filet avec 6 de marge, la vis en depasse de 10 ; 25 N.m. Pas d ecrou a bague polyamide (ISO 7040, DIN 985) : elle ne freine plus a 150 C. Acier, pas inox : meme dilatation que les flancs, la precharge tient a chaud</t>
+          <t>entretoises de cadre : 4 de coin, 2 de bielle, 1 de sommet. Serrage 80, filetage total : la vis depasse de l ecrou de 10 ; 25 N.m. Pas d ecrou a bague polyamide (ISO 7040, DIN 985) : elle ne freine plus a 150 C. Acier, pas inox : meme dilatation que les flancs, la precharge tient a chaud</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Vis H M10 x 80 ISO 4017 8.8 zinguee (filetage total) + ecrou ISO 7042 classe 8, autofreine tout metal + 2 rondelles ISO 7089 M10</t>
+          <t>Vis TH M10 x 100 ISO 4017 8.8 zinguee (filetage total) + ecrou ISO 7042 classe 8, autofreine tout metal + 2 rondelles ISO 7089 M10 : MEME ARTICLE QUE V1</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>paquet de plaques de traverse, a y = +/- 17 : les deux vis tiennent les plaques alignees pour dresser le chant en paquet ; elles ne reprennent aucune charge. Serrage 52, la vis depasse de l ecrou de 18 ; 25 N.m. Tole mesuree au dela de 10,5 : prendre des M10 x 90 (verifie() le signale)</t>
+          <t>paquet de plaques de traverse, a y = +/- 17 : les deux vis tiennent les plaques alignees pour dresser le chant en paquet ; elles ne reprennent aucune charge. Serrage 52, la vis depasse de l ecrou de 38, entre les flancs ; 25 N.m</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Butee de la vis de commande : 2 rondelles AS 1730 graissees au lieu de la butee a aiguilles
Couple de manoeuvre 14,5 N.m (frottement sous tete compte).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -1347,7 +1347,7 @@
         </is>
       </c>
       <c r="F5" s="7" t="n">
-        <v>0.353</v>
+        <v>0.345</v>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
@@ -1425,7 +1425,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Masse du cadre complet : 34.4 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 07/10/2026).</t>
+          <t>Masse du cadre complet : 34.3 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 08/10/2026).</t>
         </is>
       </c>
     </row>
@@ -1587,15 +1587,15 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Butee a aiguilles AXK 1730 + 2 rondelles AS 1730</t>
+          <t>Rondelle trempee AS 1730 (17 x 30 x 1) : MEME ARTICLE QUE V5</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>face EXTERIEURE des platines : c est elle qui encaisse les 5.5 kN de commande</t>
+          <t>sous la tete de la vis de commande, face EXTERIEURE des platines : elles encaissent les 5.5 kN de commande ; pate graphite haute temperature entre elles, la tete tourne dessus</t>
         </is>
       </c>
     </row>
@@ -2225,7 +2225,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>9.4 N.m</t>
+          <t>14.5 N.m</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Sous-ensemble de chape, sur l etabli. Sur la vis H M16 x 160 (02d), enfiler sous la tete une rondelle AS, la butee AXK 1730 et la seconde AS (V6), les deux platines, les deux rondelles trempees (V5), puis visser les deux ecrous HM (V7) : 0,1 a 0,3 mm de jeu axial, contre-bloquer. Pate cuivre sur le filet de la vis.</t>
+          <t>Sous-ensemble de chape, sur l etabli. Sur la vis H M16 x 160 (02d), enfiler sous la tete les deux rondelles AS (V6), pate graphite entre elles, les deux platines, les deux rondelles trempees (V5), puis visser les deux ecrous HM (V7) : 0,1 a 0,3 mm de jeu axial, contre-bloquer. Pate cuivre sur le filet de la vis.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Conges interieurs R2 minimum partout (controle automatique), un PDF par feuille
Coin : rebords de 4 sous conge R2, plaquettes 38 x 102/104 x 6, jeu 2 par bout.
Pied : fond des fentes de calage a degagements R2. Crochet : fond de gorge R2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="F4" s="7" t="n">
-        <v>10.206</v>
+        <v>10.201</v>
       </c>
       <c r="G4" s="7">
         <f>C4*F4</f>
@@ -855,11 +855,11 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>plat 65 x 45, L 120 (fini 61 x 40 x 114,5)</t>
+          <t>plat 70 x 45, L 120 (fini 63 x 40 x 114,5)</t>
         </is>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1.371</v>
+        <v>1.374</v>
       </c>
       <c r="G9" s="7">
         <f>C9*F9</f>
@@ -867,7 +867,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>acier taraude M16 sur 80 depuis le bout EPAIS, passage 18 au dela ; porte les deux plaques de frottement en bronze entre rebords de 3 : dessus 5,25, dessous 5,41 (faces normales a la pente)</t>
+          <t>acier taraude M16 sur 80 depuis le bout EPAIS, passage 18 au dela ; porte les deux plaques de frottement en bronze entre rebords de 4 : dessus 4,25, dessous 4,43 (faces normales a la pente)</t>
         </is>
       </c>
     </row>
@@ -892,11 +892,11 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>plat 40 x 6</t>
+          <t>plat 40 x 8</t>
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>0.171</v>
+        <v>0.205</v>
       </c>
       <c r="G10" s="7">
         <f>C10*F10</f>
@@ -904,7 +904,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>fraisee 38 x 102 x 5, sans trou, faces planes et paralleles a 0,02, Ra 0,8 cote glissement, aretes cassees 0,3 ; entre ses deux rebords sur le dessus du coin, points de silicone HT au montage ; pate graphite haute temperature sur la face qui glisse sous la traverse</t>
+          <t>fraisee 38 x 102 x 6, sans trou, faces planes et paralleles a 0,02, Ra 0,8 cote glissement, aretes cassees 0,3 ; entre ses deux rebords sur le dessus du coin, points de silicone HT au montage ; pate graphite haute temperature sur la face qui glisse sous la traverse</t>
         </is>
       </c>
     </row>
@@ -929,11 +929,11 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>plat 40 x 6</t>
+          <t>plat 40 x 8</t>
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0.174</v>
+        <v>0.209</v>
       </c>
       <c r="G11" s="7">
         <f>C11*F11</f>
@@ -941,7 +941,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>comme la haute, mais 38 x 104 x 5 ; entre ses deux rebords sous le coin, points de silicone HT au montage ; pate graphite haute temperature sur la face qui glisse sur la pente du coulisseau</t>
+          <t>comme la haute, mais 38 x 104 x 6 ; entre ses deux rebords sous le coin, points de silicone HT au montage ; pate graphite haute temperature sur la face qui glisse sur la pente du coulisseau</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="F17" s="7" t="n">
-        <v>0.87</v>
+        <v>0.868</v>
       </c>
       <c r="G17" s="7">
         <f>C17*F17</f>
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="F18" s="7" t="n">
-        <v>0.173</v>
+        <v>0.174</v>
       </c>
       <c r="G18" s="7">
         <f>C18*F18</f>
@@ -1425,7 +1425,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Masse du cadre complet : 34.3 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 09/10/2026).</t>
+          <t>Masse du cadre complet : 34.4 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 09/10/2026).</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>usinees en CuSn12-C, 38 x 102 (dessus) et 38 x 104 (dessous) x 5 ; pate graphite haute temperature ; 7.6 MPa au plus pour 25 admis</t>
+          <t>usinees en CuSn12-C, 38 x 102 (dessus) et 38 x 104 (dessous) x 6 ; pate graphite haute temperature ; 7.6 MPa au plus pour 25 admis</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>5.25 (dessus) et 5.41 (dessous) x 3, 11.8 MPa de flexion, garde 2 sous le bronze</t>
+          <t>4.25 (dessus) et 4.43 (dessous) x 4, 23.9 MPa de flexion, garde 2 sous le bronze</t>
         </is>
       </c>
     </row>
@@ -2321,7 +2321,7 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>38.0 x 50.6 mm (sur 58) en fin de course, 6.2 MPa</t>
+          <t>38.0 x 50.4 mm (sur 58) en fin de course, 6.3 MPa</t>
         </is>
       </c>
     </row>
@@ -2783,7 +2783,7 @@
     <row r="32">
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Les plats, les patins d appui et le patin de charge sont colles sur la poutrelle et partent avec elle : il faut un jeu neuf par eprouvette (4 patins d appui, 1 patin de charge, 2 plats ; colle). Le poussoir visse porte sur le patin de charge, centre par le tourillon, et la tete ne peut remonter que de 9,9 avant que le coulisseau touche les entretoises de chape : l eprouvette ne sort pas cadre ferme, on rouvre le flanc cote chape.</t>
+          <t>Les plats, les patins d appui et le patin de charge sont colles sur la poutrelle et partent avec elle : il faut un jeu neuf par eprouvette (4 patins d appui, 1 patin de charge, 2 plats ; colle). Le poussoir visse porte sur le patin de charge, centre par le tourillon, et la tete ne peut remonter que de 11 avant que le coulisseau touche les entretoises de chape : l eprouvette ne sort pas cadre ferme, on rouvre le flanc cote chape.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
R2 mini seulement sur les pieces fraisees : pieds et crochets revenus a leurs conges laser
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="F17" s="7" t="n">
-        <v>0.868</v>
+        <v>0.87</v>
       </c>
       <c r="G17" s="7">
         <f>C17*F17</f>
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="F18" s="7" t="n">
-        <v>0.174</v>
+        <v>0.173</v>
       </c>
       <c r="G18" s="7">
         <f>C18*F18</f>

</xml_diff>

<commit_message>
Toles sans chanfrein au modele 3D ni sur les plans : aretes ebavurees
Les calculs gardent 0,8 non portant a chaque bord par prudence.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -557,7 +557,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Finition des flancs** : apres decoupe et aretes cassees : SABLAGE corindon des deux faces a l identique, pression moderee (planeite), puis BRUNISSAGE noir (oxydation a chaud), aspect mat ; degraisser l huile de sortie de bain, puis film d huile ESTER synthetique haute temperature passe au chiffon et ESSUYE ; ni huile minerale ni silicone ; graduation gravee a 0.2 de profondeur au moins, traits repasses a la peinture blanche haute temperature apres brunissage. Noir mat pour la correlation d images, et quasi sans epaisseur : ni les jeux des encoches ni les serrages des entretoises n en dependent. Les autres pieces restent brutes.</t>
+          <t>Finition des flancs** : apres decoupe et ebavurage : SABLAGE corindon des deux faces a l identique, pression moderee (planeite), puis BRUNISSAGE noir (oxydation a chaud), aspect mat ; degraisser l huile de sortie de bain, puis film d huile ESTER synthetique haute temperature passe au chiffon et ESSUYE ; ni huile minerale ni silicone ; graduation gravee a 0.2 de profondeur au moins, traits repasses a la peinture blanche haute temperature apres brunissage. Noir mat pour la correlation d images, et quasi sans epaisseur : ni les jeux des encoches ni les serrages des entretoises n en dependent. Les autres pieces restent brutes.</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="F4" s="7" t="n">
-        <v>10.201</v>
+        <v>10.242</v>
       </c>
       <c r="G4" s="7">
         <f>C4*F4</f>
@@ -682,7 +682,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>decoupe laser, aretes cassees 0,8 x 45 deg, bossages non repris ; encoches a mi-bois et mortaise taillees sur la tole REELLE S355 des pieces qu elles recoivent : mesurer les deux toles livrees, regler EP_TOLE_REELLE_42 (42CrMo4) et EP_TOLE_REELLE_S355 (S355JR) et regenerer les DXF avant decoupe ; graduation de charge gravee (calque GRAVURE) d un seul cote de la lumiere, face gravee montee a l exterieur ; finition : apres decoupe et aretes cassees : SABLAGE corindon des deux faces a l identique, pression moderee (planeite), puis BRUNISSAGE noir (oxydation a chaud), aspect mat ; degraisser l huile de sortie de bain, puis film d huile ESTER synthetique haute temperature passe au chiffon et ESSUYE ; ni huile minerale ni silicone ; graduation gravee a 0.2 de profondeur au moins, traits repasses a la peinture blanche haute temperature apres brunissage</t>
+          <t>decoupe laser, aretes ebavurees (pas de chanfrein), bossages non repris ; encoches a mi-bois et mortaise taillees sur la tole REELLE S355 des pieces qu elles recoivent : mesurer les deux toles livrees, regler EP_TOLE_REELLE_42 (42CrMo4) et EP_TOLE_REELLE_S355 (S355JR) et regenerer les DXF avant decoupe ; graduation de charge gravee (calque GRAVURE) d un seul cote de la lumiere, face gravee montee a l exterieur ; finition : apres decoupe et ebavurage : SABLAGE corindon des deux faces a l identique, pression moderee (planeite), puis BRUNISSAGE noir (oxydation a chaud), aspect mat ; degraisser l huile de sortie de bain, puis film d huile ESTER synthetique haute temperature passe au chiffon et ESSUYE ; ni huile minerale ni silicone ; graduation gravee a 0.2 de profondeur au moins, traits repasses a la peinture blanche haute temperature apres brunissage</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="F5" s="7" t="n">
-        <v>0.25</v>
+        <v>0.252</v>
       </c>
       <c r="G5" s="7">
         <f>C5*F5</f>
@@ -748,7 +748,7 @@
         </is>
       </c>
       <c r="F6" s="7" t="n">
-        <v>0.325</v>
+        <v>0.327</v>
       </c>
       <c r="G6" s="7">
         <f>C6*F6</f>
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="F12" s="7" t="n">
-        <v>0.451</v>
+        <v>0.454</v>
       </c>
       <c r="G12" s="7">
         <f>C12*F12</f>
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="F14" s="7" t="n">
-        <v>0.129</v>
+        <v>0.131</v>
       </c>
       <c r="G14" s="7">
         <f>C14*F14</f>
@@ -1081,7 +1081,7 @@
         </is>
       </c>
       <c r="F15" s="7" t="n">
-        <v>0.446</v>
+        <v>0.447</v>
       </c>
       <c r="G15" s="7">
         <f>C15*F15</f>
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="F17" s="7" t="n">
-        <v>0.87</v>
+        <v>0.872</v>
       </c>
       <c r="G17" s="7">
         <f>C17*F17</f>
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="F18" s="7" t="n">
-        <v>0.173</v>
+        <v>0.174</v>
       </c>
       <c r="G18" s="7">
         <f>C18*F18</f>
@@ -1380,7 +1380,7 @@
         </is>
       </c>
       <c r="F6" s="7" t="n">
-        <v>0.26</v>
+        <v>0.264</v>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
@@ -1425,7 +1425,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Masse du cadre complet : 34.4 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 09/10/2026).</t>
+          <t>Masse du cadre complet : 34.5 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 09/10/2026).</t>
         </is>
       </c>
     </row>
@@ -2328,12 +2328,12 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Arete cassee des pieces de tole</t>
+          <t>Aretes des pieces de tole</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>0.8 x 45 degres sur les deux faces</t>
+          <t>ebavurees, sans chanfrein ; les calculs comptent 0.8 non portant a chaque bord</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plaquettes de bronze 41 de large (guident le coin dans la fente), encochees sur des tenons, fixees par 2 CHC M4 dans des oblongs
Coin : tenons 24 x 8 x 4 au milieu des bouts, conges R2 au pied, 4 taraudages M4.
Fente du coin dans les flancs ramenee a 42,2 (0,6 de jeu par cote du bronze).
Silicone supprime ; nouvelle visserie V9.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -593,7 +593,7 @@
     <col width="31" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="70" customWidth="1" min="8" max="8"/>
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="F4" s="7" t="n">
-        <v>10.242</v>
+        <v>10.25</v>
       </c>
       <c r="G4" s="7">
         <f>C4*F4</f>
@@ -855,7 +855,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>plat 70 x 45, L 120 (fini 63 x 40 x 114,5)</t>
+          <t>plat 70 x 45, L 120 (fini 63,3 x 40 x 114,5)</t>
         </is>
       </c>
       <c r="F9" s="7" t="n">
@@ -867,7 +867,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>acier taraude M16 sur 80 depuis le bout EPAIS, passage 18 au dela ; porte les deux plaques de frottement en bronze entre rebords de 4 : dessus 4,25, dessous 4,43 (faces normales a la pente)</t>
+          <t>acier taraude M16 sur 80 depuis le bout EPAIS, passage 18 au dela ; porte les deux plaques de frottement en bronze, tenons de 4 de haut et 24 de large : dessus 8, dessous 7,83 (faces normales a la pente) ; 4 taraudages M4 prof. 10 pour les vis des plaquettes</t>
         </is>
       </c>
     </row>
@@ -892,11 +892,11 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>plat 40 x 8</t>
+          <t>plat 45 x 8</t>
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>0.205</v>
+        <v>0.208</v>
       </c>
       <c r="G10" s="7">
         <f>C10*F10</f>
@@ -904,7 +904,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>fraisee 38 x 102 x 6, sans trou, faces planes et paralleles a 0,02, Ra 0,8 cote glissement, aretes cassees 0,3 ; entre ses deux rebords sur le dessus du coin, points de silicone HT au montage ; pate graphite haute temperature sur la face qui glisse sous la traverse</t>
+          <t>fraisee 41 x 114 x 6, encochee aux deux bouts autour des tenons du coin, 2 oblongs lames pour CHC M4 ; faces planes et paralleles a 0,02, Ra 0,8 cote glissement, aretes cassees 0,3 ; deborde du coin de 0,5 de chaque cote : c est elle qui touche la fente des flancs ; pate graphite haute temperature sur la face qui glisse sous la traverse</t>
         </is>
       </c>
     </row>
@@ -929,11 +929,11 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>plat 40 x 8</t>
+          <t>plat 45 x 8</t>
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0.209</v>
+        <v>0.214</v>
       </c>
       <c r="G11" s="7">
         <f>C11*F11</f>
@@ -941,7 +941,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>comme la haute, mais 38 x 104 x 6 ; entre ses deux rebords sous le coin, points de silicone HT au montage ; pate graphite haute temperature sur la face qui glisse sur la pente du coulisseau</t>
+          <t>comme la haute, mais 41 x 117 x 6, lamages cote coulisseau ; pate graphite haute temperature sur la face qui glisse sur la pente du coulisseau</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Masse du cadre complet : 34.5 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 09/10/2026).</t>
+          <t>Masse du cadre complet : 34.6 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 19/10/2026).</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1636,6 +1636,26 @@
       <c r="D11" s="6" t="inlineStr">
         <is>
           <t>vis de chape : tete et 1 rondelle derriere le flanc oppose, flanc, entretoise de cadre, flanc, entretoise de butee, platines, 4 rondelles, ecrou serre puis contre-ecrou bloque contre lui. Serrage 173,5, filet a partir de 168 : le premier ecrou y tombe avec 5,5 de marge, la vis depasse du contre-ecrou de 9,7 ; 25 N.m sur le premier</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>V9</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Vis CHC M4 x 8 ISO 4762 8.8 zinguee, tete normale</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>2 par plaque de frottement, dans ses oblongs, tete dans le lamage (0,5 sous la surface de glissement), 6,5 de filet dans les taraudages M4 du coin ; serrage LEGER, la plaquette doit glisser</t>
         </is>
       </c>
     </row>
@@ -2285,19 +2305,19 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>usinees en CuSn12-C, 38 x 102 (dessus) et 38 x 104 (dessous) x 6 ; pate graphite haute temperature ; 7.6 MPa au plus pour 25 admis</t>
+          <t>usinees en CuSn12-C, 41 x 114 (dessus) et 41 x 117 (dessous) x 6 ; pate graphite haute temperature ; 7.4 MPa au plus pour 25 admis</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Rebords des plaquettes</t>
+          <t>Tenons du coin</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>4.25 (dessus) et 4.43 (dessous) x 4, 23.9 MPa de flexion, garde 2 sous le bronze</t>
+          <t>24 x 8 x 4 de haut, conge de pied R2, 11.2 MPa de flexion, 30 MPa de matage, garde 2 sous le bronze</t>
         </is>
       </c>
     </row>
@@ -2309,7 +2329,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>30.0 x 52.8 mm (sur 60) en fin de course, 7.6 MPa</t>
+          <t>33.0 x 49.0 mm (sur 60) en fin de course, 7.4 MPa</t>
         </is>
       </c>
     </row>
@@ -2321,7 +2341,7 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>38.0 x 50.4 mm (sur 58) en fin de course, 6.3 MPa</t>
+          <t>41.0 x 47.0 mm (sur 58) en fin de course, 6.2 MPa</t>
         </is>
       </c>
     </row>
@@ -2562,7 +2582,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Coin, a l avance. Degraisser les deux sieges ; poser chaque plaque de frottement ENTRE SES DEUX REBORDS (la plus longue, 104, dessous), quelques points de silicone haute temperature sur le siege degraisse -- PAS d epoxy, bronze et acier ne se dilatent pas pareil ; laisser prendre. PUIS seulement, pate graphite haute temperature sur les faces de glissement, rien sur les sieges : le silicone ne prend pas sur une pate.</t>
+          <t>Coin, a l avance. Poser chaque plaque de frottement, encoches sur les tenons (la plus longue, 117, dessous), et la tenir par ses deux vis V9 dans leurs oblongs, SANS les bloquer : la plaquette doit glisser sous les tetes (pate a l eau sur le filet, ou une goutte de frein-filet faible). PAS de colle : bronze et acier ne se dilatent pas pareil. Puis pate graphite haute temperature sur les faces de glissement, rien sur les sieges.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fente du coin des flancs remise a 44 : seuls le coin et les plaquettes changent
Le bronze a 1,5 de jeu par cote dans la fente ; au pire des decalages, son bord
arrive au ras du bord de la traverse.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="F4" s="7" t="n">
-        <v>10.25</v>
+        <v>10.242</v>
       </c>
       <c r="G4" s="7">
         <f>C4*F4</f>
@@ -1425,7 +1425,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Masse du cadre complet : 34.6 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 19/10/2026).</t>
+          <t>Masse du cadre complet : 34.5 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 20/10/2026).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plaquettes rallongees (124 / 127) : toujours engagees dans la fente des deux flancs
Depassement de 4,75 a chaque bout du coin, borne par les ecrous interieurs de
la vis en fin de course (controle ajoute) ; engagement mini 3,75 dans la tole.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>0.208</v>
+        <v>0.215</v>
       </c>
       <c r="G10" s="7">
         <f>C10*F10</f>
@@ -904,7 +904,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>fraisee 41 x 114 x 6, encochee aux deux bouts autour des tenons du coin, 2 oblongs lames pour CHC M4 ; faces planes et paralleles a 0,02, Ra 0,8 cote glissement, aretes cassees 0,3 ; deborde du coin de 0,5 de chaque cote : c est elle qui touche la fente des flancs ; pate graphite haute temperature sur la face qui glisse sous la traverse</t>
+          <t>fraisee 41 x 124 x 6, encochee aux deux bouts autour des tenons du coin, 2 oblongs lames pour CHC M4 ; faces planes et paralleles a 0,02, Ra 0,8 cote glissement, aretes cassees 0,3 ; deborde du coin de 0,5 de chaque cote : c est elle qui touche la fente des flancs ; pate graphite haute temperature sur la face qui glisse sous la traverse</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0.214</v>
+        <v>0.221</v>
       </c>
       <c r="G11" s="7">
         <f>C11*F11</f>
@@ -941,7 +941,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>comme la haute, mais 41 x 117 x 6, lamages cote coulisseau ; pate graphite haute temperature sur la face qui glisse sur la pente du coulisseau</t>
+          <t>comme la haute, mais 41 x 127 x 6, lamages cote coulisseau ; pate graphite haute temperature sur la face qui glisse sur la pente du coulisseau</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>usinees en CuSn12-C, 41 x 114 (dessus) et 41 x 117 (dessous) x 6 ; pate graphite haute temperature ; 7.4 MPa au plus pour 25 admis</t>
+          <t>usinees en CuSn12-C, 41 x 124 (dessus) et 41 x 127 (dessous) x 6 ; pate graphite haute temperature ; 7.4 MPa au plus pour 25 admis</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Coin, a l avance. Poser chaque plaque de frottement, encoches sur les tenons (la plus longue, 117, dessous), et la tenir par ses deux vis V9 dans leurs oblongs, SANS les bloquer : la plaquette doit glisser sous les tetes (pate a l eau sur le filet, ou une goutte de frein-filet faible). PAS de colle : bronze et acier ne se dilatent pas pareil. Puis pate graphite haute temperature sur les faces de glissement, rien sur les sieges.</t>
+          <t>Coin, a l avance. Poser chaque plaque de frottement, encoches sur les tenons (la plus longue, 127, dessous), et la tenir par ses deux vis V9 dans leurs oblongs, SANS les bloquer : la plaquette doit glisser sous les tetes (pate a l eau sur le filet, ou une goutte de frein-filet faible). PAS de colle : bronze et acier ne se dilatent pas pareil. Puis pate graphite haute temperature sur les faces de glissement, rien sur les sieges.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plaquettes 133 / 136 : engagees sur toute l'epaisseur des deux flancs ; visionneuse 3D avec course du coin
Les branches des plaquettes passent de part et d'autre des ecrous V7 (controle
corrige). Visionneuse : curseur de course, coulisseau, pile ecrasee, effort, butee.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>0.215</v>
+        <v>0.221</v>
       </c>
       <c r="G10" s="7">
         <f>C10*F10</f>
@@ -904,7 +904,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>fraisee 41 x 124 x 6, encochee aux deux bouts autour des tenons du coin, 2 oblongs lames pour CHC M4 ; faces planes et paralleles a 0,02, Ra 0,8 cote glissement, aretes cassees 0,3 ; deborde du coin de 0,5 de chaque cote : c est elle qui touche la fente des flancs ; pate graphite haute temperature sur la face qui glisse sous la traverse</t>
+          <t>fraisee 41 x 133 x 6, encochee aux deux bouts autour des tenons du coin, 2 oblongs lames pour CHC M4 ; faces planes et paralleles a 0,02, Ra 0,8 cote glissement, aretes cassees 0,3 ; deborde du coin de 0,5 de chaque cote : c est elle qui touche la fente des flancs ; pate graphite haute temperature sur la face qui glisse sous la traverse</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0.221</v>
+        <v>0.227</v>
       </c>
       <c r="G11" s="7">
         <f>C11*F11</f>
@@ -941,7 +941,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>comme la haute, mais 41 x 127 x 6, lamages cote coulisseau ; pate graphite haute temperature sur la face qui glisse sur la pente du coulisseau</t>
+          <t>comme la haute, mais 41 x 136 x 6, lamages cote coulisseau ; pate graphite haute temperature sur la face qui glisse sur la pente du coulisseau</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Masse du cadre complet : 34.5 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 20/10/2026).</t>
+          <t>Masse du cadre complet : 34.6 kg. Poutrelle beton : 22.2 kg. Masses du modele 3D (out/masses.json du 20/10/2026).</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>usinees en CuSn12-C, 41 x 124 (dessus) et 41 x 127 (dessous) x 6 ; pate graphite haute temperature ; 7.4 MPa au plus pour 25 admis</t>
+          <t>usinees en CuSn12-C, 41 x 133 (dessus) et 41 x 136 (dessous) x 6 ; pate graphite haute temperature ; 7.4 MPa au plus pour 25 admis</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Coin, a l avance. Poser chaque plaque de frottement, encoches sur les tenons (la plus longue, 127, dessous), et la tenir par ses deux vis V9 dans leurs oblongs, SANS les bloquer : la plaquette doit glisser sous les tetes (pate a l eau sur le filet, ou une goutte de frein-filet faible). PAS de colle : bronze et acier ne se dilatent pas pareil. Puis pate graphite haute temperature sur les faces de glissement, rien sur les sieges.</t>
+          <t>Coin, a l avance. Poser chaque plaque de frottement, encoches sur les tenons (la plus longue, 136, dessous), et la tenir par ses deux vis V9 dans leurs oblongs, SANS les bloquer : la plaquette doit glisser sous les tetes (pate a l eau sur le filet, ou une goutte de frein-filet faible). PAS de colle : bronze et acier ne se dilatent pas pareil. Puis pate graphite haute temperature sur les faces de glissement, rien sur les sieges.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plaquettes : branches reliees par un pont (fenetre autour des tenons), angles en conge R2
Le pont de la plaquette basse atteint les ecrous V7 au dela de 53,2 mm de course
(sur 55,5) : accepte, signale dans le bilan de params.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>0.221</v>
+        <v>0.24</v>
       </c>
       <c r="G10" s="7">
         <f>C10*F10</f>
@@ -904,7 +904,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>fraisee 41 x 133 x 6, encochee aux deux bouts autour des tenons du coin, 2 oblongs lames pour CHC M4 ; faces planes et paralleles a 0,02, Ra 0,8 cote glissement, aretes cassees 0,3 ; deborde du coin de 0,5 de chaque cote : c est elle qui touche la fente des flancs ; pate graphite haute temperature sur la face qui glisse sous la traverse</t>
+          <t>fraisee 41 x 133 x 6, une fenetre a chaque bout autour des tenons du coin, 2 oblongs lames pour CHC M4 ; faces planes et paralleles a 0,02, Ra 0,8 cote glissement, aretes cassees 0,3 ; deborde du coin de 0,5 de chaque cote : c est elle qui touche la fente des flancs ; pate graphite haute temperature sur la face qui glisse sous la traverse</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0.227</v>
+        <v>0.247</v>
       </c>
       <c r="G11" s="7">
         <f>C11*F11</f>

</xml_diff>

<commit_message>
Coin : pied des tenons vif (outil vertical), fenetres des plaquettes resserrees a 0,5 ; taraudages M4 en traits caches sur la vue de face
Fenetre de la plaquette basse elargie au bout epais de H.tan(a) : la face de
bout du tenon y est verticale.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1.374</v>
+        <v>1.372</v>
       </c>
       <c r="G9" s="7">
         <f>C9*F9</f>
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>0.24</v>
+        <v>0.254</v>
       </c>
       <c r="G10" s="7">
         <f>C10*F10</f>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0.247</v>
+        <v>0.259</v>
       </c>
       <c r="G11" s="7">
         <f>C11*F11</f>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>usinees en CuSn12-C, 41 x 133 (dessus) et 41 x 136 (dessous) x 6 ; pate graphite haute temperature ; 7.4 MPa au plus pour 25 admis</t>
+          <t>usinees en CuSn12-C, 41 x 133 (dessus) et 41 x 136 (dessous) x 6 ; pate graphite haute temperature ; 7.2 MPa au plus pour 25 admis</t>
         </is>
       </c>
     </row>
@@ -2317,7 +2317,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>24 x 8 x 4 de haut, conge de pied R2, 11.2 MPa de flexion, 30 MPa de matage, garde 2 sous le bronze</t>
+          <t>24 x 8 x 4 de haut, pied vif (outil vertical), 11.2 MPa de flexion, 15 MPa de matage, garde 2 sous le bronze</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>33.0 x 49.0 mm (sur 60) en fin de course, 7.4 MPa</t>
+          <t>33.0 x 50.5 mm (sur 60) en fin de course, 7.2 MPa</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>41.0 x 47.0 mm (sur 58) en fin de course, 6.2 MPa</t>
+          <t>41.0 x 48.4 mm (sur 58) en fin de course, 6.0 MPa</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plaquettes : conge R4 sur le pourtour de la face de glissement (rayon de la fente du flanc), angles en plan R4 ; pressions sur 33 portants
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/NOMENCLATURE.xlsx
+++ b/out/NOMENCLATURE.xlsx
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>0.254</v>
+        <v>0.243</v>
       </c>
       <c r="G10" s="7">
         <f>C10*F10</f>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0.259</v>
+        <v>0.249</v>
       </c>
       <c r="G11" s="7">
         <f>C11*F11</f>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>usinees en CuSn12-C, 41 x 133 (dessus) et 41 x 136 (dessous) x 6 ; pate graphite haute temperature ; 7.2 MPa au plus pour 25 admis</t>
+          <t>usinees en CuSn12-C, 41 x 133 (dessus) et 41 x 136 (dessous) x 6 ; pate graphite haute temperature ; 9.5 MPa au plus pour 25 admis</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>33.0 x 50.5 mm (sur 60) en fin de course, 7.2 MPa</t>
+          <t>25.0 x 50.5 mm (sur 60) en fin de course, 9.5 MPa</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>41.0 x 48.4 mm (sur 58) en fin de course, 6.0 MPa</t>
+          <t>41.0 x 48.4 mm (sur 58) en fin de course, 7.5 MPa</t>
         </is>
       </c>
     </row>

</xml_diff>